<commit_message>
chore: finalize unicef submission docs and team additions
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_DataPlan.xlsx
+++ b/Galeon_UNICEF_DataPlan.xlsx
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F11" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza (Co-founder, technical lead)</t>
+          <t>Mateo Daza (technical lead) + Juan David Correa (project coordination)</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F15" s="45" t="inlineStr">
         <is>
-          <t>Fabio Anaya (UNICEF partnership lead) + Mateo Daza</t>
+          <t>Fabio Anaya (Growth lead) + Mateo Daza + Juan David Correa (project coordination)</t>
         </is>
       </c>
     </row>
@@ -1284,22 +1284,22 @@
       </c>
       <c r="B19" s="45" t="inlineStr">
         <is>
-          <t>Embedded email-based wallet onboarding (Privy)</t>
+          <t>Beneficiary onboarding — embedded email-based wallet (Privy) + account abstraction</t>
         </is>
       </c>
       <c r="C19" s="45" t="inlineStr">
         <is>
-          <t>First-time users can receive a wallet via email login; no seed phrases shown. Recovery via email is documented and tested.</t>
+          <t>First-time users receive a wallet via email login, never see seed phrases, and do not pay or manage gas fees. Account abstraction enables partner-sponsored gas, batched operations, and email/social recovery. The goal: a beneficiary opens a link, logs in, receives stablecoins — and does not need to know they are using crypto until they have the balance. Mobile-first design throughout (most beneficiaries access via phone).</t>
         </is>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
-          <t>End-to-end flow: invite link → email login → first stablecoin payment received, completed in &lt;5 minutes by a non-crypto tester.</t>
+          <t>End-to-end flow on mobile: invite link → email login → first stablecoin payment received, completed in &lt;5 minutes by a non-crypto tester. Gas sponsored by partner; no seed phrase shown.</t>
         </is>
       </c>
       <c r="E19" s="45" t="inlineStr">
         <is>
-          <t>Frontend code (apps/web/app/setup), test recordings with consent, task-completion metrics.</t>
+          <t>Frontend code (apps/web/app/setup), test recordings with consent, mobile-flow task-completion metrics, partner-sponsor gas configuration.</t>
         </is>
       </c>
       <c r="F19" s="45" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B20" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Integrate Privy embedded-wallet SDK with email recovery into the Setup flow.</t>
+          <t>Activity 1 — Integrate Privy embedded-wallet SDK with email recovery and account abstraction (smart wallet, gas sponsorship hooks) into the Setup flow.</t>
         </is>
       </c>
       <c r="C20" s="46" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B21" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Lightweight redesign of Setup, Receive, Pay, and Collect for non-technical first-time users (clearer copy, larger CTAs, illustrated steps). No multi-language work in Q1.</t>
+          <t>Activity 2 — Mobile-first redesign of Setup, Receive, Pay, and Collect for non-technical first-time users on smartphones (large touch targets, clear copy, illustrated steps, no crypto jargon visible).</t>
         </is>
       </c>
       <c r="C21" s="46" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="F39" s="45" t="inlineStr">
         <is>
-          <t>Carlos Quintero + Mateo Daza</t>
+          <t>Carlos Quintero + Mateo Daza + Juan David Correa (remediation tracking)</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="F47" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza</t>
+          <t>Mateo Daza + Juan José Sanfeliú (community engagement)</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="F49" s="46" t="inlineStr">
         <is>
-          <t>Mateo Daza</t>
+          <t>Mateo Daza + Juan José Sanfeliú (announcement, community engagement)</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="F51" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + Fabio Anaya + partner program officer</t>
+          <t>Mateo Daza + Fabio Anaya + Juan David Correa (runbook + coordination) + partner program officer</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="F62" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + Fabio Anaya + partner program officer</t>
+          <t>Mateo Daza + Fabio Anaya + Juan David Correa (project coordination) + partner program officer</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="F96" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza</t>
+          <t>Mateo Daza + Juan José Sanfeliú (developer relations and content)</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="F98" s="46" t="inlineStr">
         <is>
-          <t>Mateo Daza + Carlos Quintero</t>
+          <t>Mateo Daza + Carlos Quintero + Juan José Sanfeliú (developer outreach)</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="F100" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + Carlos Quintero</t>
+          <t>Mateo Daza + Fabio Anaya (partner engagement) + Juan José Sanfeliú (communications)</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="F102" s="46" t="inlineStr">
         <is>
-          <t>Mateo Daza</t>
+          <t>Fabio Anaya + Juan José Sanfeliú + Mateo Daza</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       <c r="A121" s="13" t="n"/>
       <c r="B121" s="50" t="inlineStr">
         <is>
-          <t>4. Embedded email-based wallet onboarding (Privy) for non-crypto-literate beneficiaries.</t>
+          <t>4. Embedded email-based wallet (Privy) + account abstraction + mobile-first UX for non-crypto-literate beneficiaries (no seed phrases, no gas, mobile-optimised).</t>
         </is>
       </c>
       <c r="C121" s="17" t="n"/>
@@ -3602,7 +3602,7 @@
       <c r="A125" s="13" t="n"/>
       <c r="B125" s="50" t="inlineStr">
         <is>
-          <t>(iii) Embedded-wallet onboarding integration + low-literacy UI components — MIT.</t>
+          <t>(iii) Embedded-wallet + account-abstraction onboarding integration and mobile-first low-literacy UI components — MIT.</t>
         </is>
       </c>
       <c r="C125" s="17" t="n"/>

</xml_diff>

<commit_message>
docs: finalize UNICEF submission documents
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_DataPlan.xlsx
+++ b/Galeon_UNICEF_DataPlan.xlsx
@@ -977,7 +977,7 @@
       </c>
       <c r="C7" s="45" t="inlineStr">
         <is>
-          <t>Repo verifiably trustworthy: CI fails on test failures, coverage reports published, and the ERC-20 (stablecoin) pool deployed to mainnet — the version actually relevant to humanitarian cash transfers.</t>
+          <t>Repo verifiably trustworthy: CI test masking corrected pre-submission; coverage reports published; ERC-20 (stablecoin) pool deployed and verified on the current production chain to validate the implementation in production. Pilot deployment chain is confirmed separately during partner scoping (Milestone 3); if different from the current chain, redeployment to the pilot chain is part of Q2 pre-pilot preparation.</t>
         </is>
       </c>
       <c r="D7" s="45" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B9" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Deploy GaleonPrivacyPoolComplex (ERC-20) to mainnet for USDC and USDT; integrate with Entrypoint; run end-to-end deposit + withdrawal test against live contracts.</t>
+          <t>Activity 2 — Deploy GaleonPrivacyPoolComplex (ERC-20) to mainnet on the current production chain for USDC and USDT; integrate with Entrypoint; run end-to-end deposit + withdrawal test against live contracts.</t>
         </is>
       </c>
       <c r="C9" s="46" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B17" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Convert top-ranked organisation into a signed LOI scoped to a ≤50-beneficiary Q3 controlled pilot. Draft operational dependency model with the partner: KYC (partner), off-ramp/cash-out (partner + licensed provider), lost-access/SIM-swap recovery (Privy + partner), liquidity (partner), sanctions false-positive appeals (Galeon ASP policy), beneficiary support (partner).</t>
+          <t>Activity 2 — Convert top-ranked organisation into a signed LOI scoped to a ≤50-beneficiary Q3 controlled pilot. Draft operational dependency model with the partner: KYC (partner), off-ramp/cash-out (partner + licensed provider), lost-access/SIM-swap recovery (Privy + partner), liquidity (partner), sanctions false-positive appeals (Galeon ASP policy), beneficiary support (partner), pilot deployment chain (jointly confirmed based on partner geography and deployment constraints).</t>
         </is>
       </c>
       <c r="C17" s="46" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B31" s="47" t="inlineStr">
         <is>
-          <t>Backend: ERC-20 stablecoin pool deployed and verified on Mantle Mainnet. CI hardened (no `|| true`). Coverage report published. Audit engaged with frozen branch. One LOI from prospective pilot partner.</t>
+          <t>Backend: ERC-20 stablecoin pool deployed and verified to mainnet on the current production chain (implementation validation; pilot deployment chain confirmed during partner scoping). CI hardened (no `|| true`). Coverage report published. Audit engaged with frozen branch. One LOI from prospective pilot partner.</t>
         </is>
       </c>
       <c r="C31" s="47" t="inlineStr">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="C35" s="45" t="inlineStr">
         <is>
-          <t>The ASP service stops auto-approving every deposit. New approval pipeline checks each deposit label against a sanctions list (e.g., OFAC SDN) and a project-maintained blocklist; rejected labels are publicly logged.</t>
+          <t>The ASP service stops auto-approving every deposit. New approval pipeline screens each deposit label (the Port-approving address — not beneficiary identity, amounts, or any personal data) against a sanctions list (e.g., OFAC SDN) and a project-maintained blocklist. The ASP runs on a weekly attestation cadence, operated by Galeon under Cartagena On Chain (single operator during the funded period; multi-operator decentralisation is a long-term roadmap item, not in scope). Rejected labels are publicly logged via IPFS-published attestation trees. Beneficiary protection (false-positive case): no deposited funds are locked — the affected depositor recovers funds via a public ragequit withdrawal to the original deposit address. They may lose private withdrawal access for that deposit, but not access to the funds.</t>
         </is>
       </c>
       <c r="D35" s="45" t="inlineStr">
         <is>
-          <t>Production ASP rejects at least one test-injected sanctioned address; published ASP policy document; first IPFS-published attestation tree.</t>
+          <t>Production ASP rejects at least one test-injected sanctioned address; published ASP policy document including appeals process and manual-review SLA; first 5 weekly attestation trees published to IPFS with CIDs on-chain; documented evidence of ragequit working for a test-rejected deposit.</t>
         </is>
       </c>
       <c r="E35" s="45" t="inlineStr">
         <is>
-          <t>ASP service code, screening provider integration (e.g., Chainalysis Address Screening, Elliptic Navigator), rejection logs, policy doc, IPFS CID of attestation tree.</t>
+          <t>ASP service code, screening provider integration (e.g., Chainalysis Address Screening, Elliptic Navigator, or open-source OFAC SDN), rejection logs, ASP policy document, weekly attestation tree IPFS CIDs, on-chain root-update tx hashes, ragequit test transaction.</t>
         </is>
       </c>
       <c r="F35" s="45" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B36" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Select &amp; integrate a screening provider (Chainalysis / Elliptic / TRM Labs free tier or open-source list like OFAC SDN); design rejection-handling protocol that preserves the anonymity set for non-rejected labels.</t>
+          <t>Activity 1 — Select &amp; integrate a screening provider (Chainalysis / Elliptic / TRM Labs free tier or open-source list like OFAC SDN); design rejection-handling protocol that preserves the anonymity set for non-rejected labels. Define manual-review workflow: borderline addresses flagged for review by Galeon engineering, with escalation to external legal counsel for ambiguous cases. Publish appeals process with 5-business-day SLA, allowing depositors to contest a rejection.</t>
         </is>
       </c>
       <c r="C36" s="46" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="D36" s="46" t="inlineStr">
         <is>
-          <t>Integration tests cover: (i) clean address approved, (ii) sanctioned address rejected, (iii) borderline address flagged for manual review.</t>
+          <t>Integration tests cover: (i) clean address approved, (ii) sanctioned address rejected, (iii) borderline address flagged for manual review, (iv) rejected depositor successfully ragequits and recovers funds.</t>
         </is>
       </c>
       <c r="E36" s="46" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B37" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Publish ASP policy (what is screened, how, who can appeal); start publishing ASP attestation trees on IPFS with the CID stored on-chain via the existing Entrypoint hook.</t>
+          <t>Activity 2 — Publish ASP policy (what is screened, how, who can appeal, manual-review SLA, ragequit recourse for rejected deposits); start publishing ASP attestation trees on IPFS with the CID stored on-chain via the existing Entrypoint hook on a weekly cadence.</t>
         </is>
       </c>
       <c r="C37" s="46" t="inlineStr">
@@ -1923,22 +1923,22 @@
       </c>
       <c r="B47" s="45" t="inlineStr">
         <is>
-          <t>Public open-source release (month-six commitment)</t>
+          <t>Open-source maintenance and community readiness</t>
         </is>
       </c>
       <c r="C47" s="45" t="inlineStr">
         <is>
-          <t>All Galeon code released under permissive licences (MIT for apps/libs, Apache-2.0 for contracts/pool SDK) by month six of the funded period, per UNICEF open-source requirements. CONTRIBUTING.md and CODE_OF_CONDUCT.md in place. From public GitHub release through contract end plus 12 months, Project Data will remain accessible in real time with 99% uptime.</t>
+          <t>Repository is already publicly accessible under permissive licences (MIT for apps/libs, Apache-2.0 for contracts/pool — inherited from 0xbow); the UNICEF month-six open-source requirement is met from the start of the funded period. Q2 work focuses on community readiness: security review and secrets audit on the public repo, CONTRIBUTING.md, CODE_OF_CONDUCT.md, UNICEF Innovation Fund attribution per contractual terms. From the funded-period release point through contract end plus 12 months, Project Data remains accessible in real time with 99% uptime.</t>
         </is>
       </c>
       <c r="D47" s="45" t="inlineStr">
         <is>
-          <t>Public GitHub organisation live; contribution guide and code of conduct published; secrets scan clean.</t>
+          <t>Public repository remains live throughout; contribution guide and code of conduct published; security review + secrets scan clean; UNICEF attribution applied; external contributions enabled.</t>
         </is>
       </c>
       <c r="E47" s="45" t="inlineStr">
         <is>
-          <t>Public-repo URL, CONTRIBUTING.md, CODE_OF_CONDUCT.md, TruffleHog secrets-scan report.</t>
+          <t>CONTRIBUTING.md, CODE_OF_CONDUCT.md, TruffleHog secrets-scan report, UNICEF attribution diff, repository activity log.</t>
         </is>
       </c>
       <c r="F47" s="45" t="inlineStr">
@@ -1955,17 +1955,17 @@
       </c>
       <c r="B48" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Final security review, secrets audit (TruffleHog), license-header sweep across all packages.</t>
+          <t>Activity 1 — Security review of the public repository: secrets audit (TruffleHog) to confirm no credentials leaked historically, license-header sweep across all packages, dependency vulnerability scan. Remediate any findings.</t>
         </is>
       </c>
       <c r="C48" s="46" t="inlineStr">
         <is>
-          <t>Repository cleared for public release.</t>
+          <t>Security review complete; any findings remediated.</t>
         </is>
       </c>
       <c r="D48" s="46" t="inlineStr">
         <is>
-          <t>Audit checklist completed; secrets scan clean.</t>
+          <t>Audit checklist completed; secrets scan clean; no critical vulnerabilities open.</t>
         </is>
       </c>
       <c r="E48" s="46" t="inlineStr">
@@ -1987,22 +1987,22 @@
       </c>
       <c r="B49" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Migrate monorepo to public GitHub organisation; publish announcement; archive private repo.</t>
+          <t>Activity 2 — Publish CONTRIBUTING.md, CODE_OF_CONDUCT.md, and governance notes; apply UNICEF Innovation Fund attribution to the repository per contractual terms; publish an open-source community announcement.</t>
         </is>
       </c>
       <c r="C49" s="46" t="inlineStr">
         <is>
-          <t>Public repo live; announcement published.</t>
+          <t>Contribution guides and UNICEF attribution published; community announcement live.</t>
         </is>
       </c>
       <c r="D49" s="46" t="inlineStr">
         <is>
-          <t>Public visibility on github.com.</t>
+          <t>CONTRIBUTING and CODE_OF_CONDUCT visible on github.com; UNICEF attribution diff merged.</t>
         </is>
       </c>
       <c r="E49" s="46" t="inlineStr">
         <is>
-          <t>Public-repo URL, announcement post.</t>
+          <t>CONTRIBUTING.md, CODE_OF_CONDUCT.md, attribution commit, announcement post.</t>
         </is>
       </c>
       <c r="F49" s="46" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="B52" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Set up staging environment mirroring production; create test-token faucet; prepare training materials.</t>
+          <t>Activity 1 — Set up staging environment mirroring production; if pilot deployment chain (confirmed in Q1 M3) differs from the current production chain, redeploy contracts to the pilot chain mainnet; create test-token faucet; prepare training materials.</t>
         </is>
       </c>
       <c r="C52" s="46" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B58" s="47" t="inlineStr">
         <is>
-          <t>Backend: Real ASP filtering live (sanctions + blocklist + IPFS attestation); audit closed with letter of resolution; DPIA published; repo public by month six; partner staff validated in sandbox.</t>
+          <t>Backend: Real ASP filtering live (sanctions + blocklist + IPFS attestation); audit closed with letter of resolution; DPIA published; public repository security-reviewed with UNICEF attribution applied; partner staff validated in sandbox.</t>
         </is>
       </c>
       <c r="C58" s="47" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="D58" s="47" t="inlineStr">
         <is>
-          <t>First sanctioned-address test rejection; auditor letter; DPIA published; public repo live; sandbox sign-off.</t>
+          <t>First sanctioned-address test rejection on production ASP; auditor letter; DPIA published; community readiness items live; sandbox sign-off.</t>
         </is>
       </c>
       <c r="E58" s="47" t="inlineStr">
@@ -3638,7 +3638,7 @@
       <c r="A128" s="13" t="n"/>
       <c r="B128" s="52" t="inlineStr">
         <is>
-          <t>None. Every new component developed during the UNICEF-funded period will be released under an OSI-approved permissive licence. Licensing follows the existing repo convention: MIT for applications and libraries (apps/web, apps/api, apps/indexer, packages/stealth, packages/config, packages/types, packages/eslint-config); Apache-2.0 for smart contracts and pool SDK (packages/contracts, packages/pool — inherited from 0xbow upstream). The repository will be made public by month six. The only non-public elements are: (a) operational pilot configuration data (kept private for beneficiary safety, not as IP); (b) commercial agreements with paying ASP-attestation customers (contracts, not code).</t>
+          <t>None. Every new component developed during the UNICEF-funded period will be released under an OSI-approved permissive licence. Licensing follows the existing repo convention: MIT for applications and libraries (apps/web, apps/api, apps/indexer, packages/stealth, packages/config, packages/types, packages/eslint-config); Apache-2.0 for smart contracts and pool SDK (packages/contracts, packages/pool — inherited from 0xbow upstream). The repository is already public. The only non-public elements are: (a) operational pilot configuration data (kept private for beneficiary safety, not as IP); (b) commercial agreements with paying ASP-attestation customers (contracts, not code).</t>
         </is>
       </c>
       <c r="C128" s="17" t="n"/>

</xml_diff>

<commit_message>
fix: on unicef docs
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_DataPlan.xlsx
+++ b/Galeon_UNICEF_DataPlan.xlsx
@@ -1212,12 +1212,12 @@
       </c>
       <c r="B16" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Discovery sessions with 3-5 UNICEF country offices and 2-3 NGO partners; document fit, regulatory environment, on/off-ramp availability per geography.</t>
+          <t>Activity 1 — Discovery sessions with UNICEF country offices and NGO partners; document fit, regulatory environment, on/off-ramp availability per geography.</t>
         </is>
       </c>
       <c r="C16" s="46" t="inlineStr">
         <is>
-          <t>Discovery completed with at least 5 organisations.</t>
+          <t>Discovery completed with a shortlisted set of organisations.</t>
         </is>
       </c>
       <c r="D16" s="46" t="inlineStr">
@@ -1284,17 +1284,17 @@
       </c>
       <c r="B19" s="45" t="inlineStr">
         <is>
-          <t>Beneficiary onboarding — embedded email-based wallet (Privy) + account abstraction</t>
+          <t>Beneficiary onboarding — embedded email-based wallet and gas-simplification options</t>
         </is>
       </c>
       <c r="C19" s="45" t="inlineStr">
         <is>
-          <t>First-time users receive a wallet via email login, never see seed phrases, and do not pay or manage gas fees. Account abstraction enables partner-sponsored gas, batched operations, and email/social recovery. The goal: a beneficiary opens a link, logs in, receives stablecoins — and does not need to know they are using crypto until they have the balance. Mobile-first design throughout (most beneficiaries access via phone).</t>
+          <t>Evaluate and implement wallet onboarding and gas-simplification options where supported by the selected provider (Privy or equivalent), so first-time beneficiaries do not need to manage seed phrases or gas fees. Mobile-first design throughout (most beneficiaries access via phone).</t>
         </is>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
-          <t>End-to-end flow on mobile: invite link → email login → first stablecoin payment received, completed in &lt;5 minutes by a non-crypto tester. Gas sponsored by partner; no seed phrase shown.</t>
+          <t>End-to-end flow on mobile: invite link → login → first stablecoin payment received, completed in a target window agreed with partner; no seed phrase exposed to the user.</t>
         </is>
       </c>
       <c r="E19" s="45" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B20" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Integrate Privy embedded-wallet SDK with email recovery and account abstraction (smart wallet, gas sponsorship hooks) into the Setup flow.</t>
+          <t>Activity 1 — Integrate Privy (or equivalent) embedded-wallet SDK with email recovery; evaluate gas-sponsorship options supported by the provider.</t>
         </is>
       </c>
       <c r="C20" s="46" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D21" s="46" t="inlineStr">
         <is>
-          <t>Internal review passes; 5-user pre-test shows ≥80% task completion.</t>
+          <t>Internal review passes; small pre-test (size to be defined) confirms the flow works for non-technical users.</t>
         </is>
       </c>
       <c r="E21" s="46" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="D29" s="47" t="inlineStr">
         <is>
-          <t>Internal pre-test ≥80% task completion.</t>
+          <t>Internal pre-test completed; results reviewed with partner before pilot scoping.</t>
         </is>
       </c>
       <c r="E29" s="47" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="D31" s="47" t="inlineStr">
         <is>
-          <t>Block-explorer verified contract; green CI on failures; coverage ≥80%; signed audit contract; signed LOI.</t>
+          <t>Block-explorer verified contract; green CI on failures; coverage tooling installed with a baseline report published; signed audit contract; signed LOI.</t>
         </is>
       </c>
       <c r="E31" s="47" t="inlineStr">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="C35" s="45" t="inlineStr">
         <is>
-          <t>The ASP service stops auto-approving every deposit. New approval pipeline screens each deposit label (the Port-approving address — not beneficiary identity, amounts, or any personal data) against a sanctions list (e.g., OFAC SDN) and a project-maintained blocklist. The ASP runs on a weekly attestation cadence, operated by Galeon under Cartagena On Chain (single operator during the funded period; multi-operator decentralisation is a long-term roadmap item, not in scope). Rejected labels are publicly logged via IPFS-published attestation trees. Beneficiary protection (false-positive case): no deposited funds are locked — the affected depositor recovers funds via a public ragequit withdrawal to the original deposit address. They may lose private withdrawal access for that deposit, but not access to the funds.</t>
+          <t>The ASP service stops auto-approving every deposit. New approval pipeline screens each deposit label (the Port-approving address — not beneficiary identity, amounts, or any personal data) against a sanctions list (e.g., OFAC SDN) and a project-maintained blocklist. The ASP runs on a regular attestation cadence (frequency to be defined during Q2 design), operated by Galeon under Cartagena On Chain (single operator during the funded period; multi-operator decentralisation is a long-term roadmap item, not in scope). Rejected labels are publicly logged via IPFS-published attestation trees. Beneficiary protection (false-positive case): no deposited funds are locked — the affected depositor recovers funds via a public ragequit withdrawal to the original deposit address. They may lose private withdrawal access for that deposit, but not access to the funds.</t>
         </is>
       </c>
       <c r="D35" s="45" t="inlineStr">
         <is>
-          <t>Production ASP rejects at least one test-injected sanctioned address; published ASP policy document including appeals process and manual-review SLA; first 5 weekly attestation trees published to IPFS with CIDs on-chain; documented evidence of ragequit working for a test-rejected deposit.</t>
+          <t>Production ASP rejects at least one test-injected sanctioned address; published ASP policy document including appeals process and manual-review SLA (specific duration to be defined); first attestation trees published to IPFS with CIDs on-chain; documented evidence of ragequit working for a test-rejected deposit.</t>
         </is>
       </c>
       <c r="E35" s="45" t="inlineStr">
         <is>
-          <t>ASP service code, screening provider integration (e.g., Chainalysis Address Screening, Elliptic Navigator, or open-source OFAC SDN), rejection logs, ASP policy document, weekly attestation tree IPFS CIDs, on-chain root-update tx hashes, ragequit test transaction.</t>
+          <t>ASP service code, screening provider integration (e.g., Chainalysis Address Screening, Elliptic Navigator, or open-source OFAC SDN), rejection logs, ASP policy document, attestation tree IPFS CIDs, on-chain root-update tx hashes, ragequit test transaction.</t>
         </is>
       </c>
       <c r="F35" s="45" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B36" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Select &amp; integrate a screening provider (Chainalysis / Elliptic / TRM Labs free tier or open-source list like OFAC SDN); design rejection-handling protocol that preserves the anonymity set for non-rejected labels. Define manual-review workflow: borderline addresses flagged for review by Galeon engineering, with escalation to external legal counsel for ambiguous cases. Publish appeals process with 5-business-day SLA, allowing depositors to contest a rejection.</t>
+          <t>Activity 1 — Select &amp; integrate a screening provider (Chainalysis / Elliptic / TRM Labs free tier or open-source list like OFAC SDN); design rejection-handling protocol that preserves the anonymity set for non-rejected labels. Define manual-review workflow: borderline addresses flagged for review by Galeon engineering, with escalation to external legal counsel for ambiguous cases. Publish appeals process (SLA to be defined with partner and counsel) allowing depositors to contest a rejection.</t>
         </is>
       </c>
       <c r="C36" s="46" t="inlineStr">
@@ -1675,17 +1675,17 @@
       </c>
       <c r="B37" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Publish ASP policy (what is screened, how, who can appeal, manual-review SLA, ragequit recourse for rejected deposits); start publishing ASP attestation trees on IPFS with the CID stored on-chain via the existing Entrypoint hook on a weekly cadence.</t>
+          <t>Activity 2 — Publish ASP policy (what is screened, how, who can appeal, manual-review process, ragequit recourse for rejected deposits); start publishing ASP attestation trees on IPFS with the CID stored on-chain via the existing Entrypoint hook on a regular cadence.</t>
         </is>
       </c>
       <c r="C37" s="46" t="inlineStr">
         <is>
-          <t>Policy published; first 5 weekly attestation trees on IPFS.</t>
+          <t>Policy published; first attestation trees published on IPFS.</t>
         </is>
       </c>
       <c r="D37" s="46" t="inlineStr">
         <is>
-          <t>Policy document live; on-chain root-update events include real IPFS CIDs.</t>
+          <t>Policy document live; on-chain root-update events include IPFS content identifiers.</t>
         </is>
       </c>
       <c r="E37" s="46" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="E47" s="45" t="inlineStr">
         <is>
-          <t>CONTRIBUTING.md, CODE_OF_CONDUCT.md, TruffleHog secrets-scan report, UNICEF attribution diff, repository activity log.</t>
+          <t>CONTRIBUTING.md, CODE_OF_CONDUCT.md, secrets-scan report, UNICEF attribution diff, repository activity log.</t>
         </is>
       </c>
       <c r="F47" s="45" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="B48" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Security review of the public repository: secrets audit (TruffleHog) to confirm no credentials leaked historically, license-header sweep across all packages, dependency vulnerability scan. Remediate any findings.</t>
+          <t>Activity 1 — Security review of the public repository: secrets audit to confirm no credentials leaked historically, license-header sweep across all packages, dependency vulnerability scan. Remediate any findings.</t>
         </is>
       </c>
       <c r="C48" s="46" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="E48" s="46" t="inlineStr">
         <is>
-          <t>Checklist, TruffleHog report, license-header diff.</t>
+          <t>Checklist, secrets-scan report, license-header diff.</t>
         </is>
       </c>
       <c r="F48" s="46" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="C51" s="45" t="inlineStr">
         <is>
-          <t>3-5 partner staff complete the full flow (Port creation, stablecoin deposit, ZK withdrawal, Shipwreck report) in a staging environment using test tokens. Operational runbook validated.</t>
+          <t>a small group of partner staff complete the full flow (Port creation, stablecoin deposit, ZK withdrawal, Shipwreck report) in a staging environment using test tokens. Operational runbook validated.</t>
         </is>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -2091,12 +2091,12 @@
       </c>
       <c r="B53" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Moderated sandbox sessions with 3-5 partner staff; iterate on runbook based on feedback.</t>
+          <t>Activity 2 — Moderated sandbox sessions with a small group of partner staff; iterate on runbook based on feedback.</t>
         </is>
       </c>
       <c r="C53" s="46" t="inlineStr">
         <is>
-          <t>5 sessions completed; runbook updated.</t>
+          <t>sessions completed; runbook updated.</t>
         </is>
       </c>
       <c r="D53" s="46" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="D62" s="45" t="inlineStr">
         <is>
-          <t>≥25 verified beneficiary transactions; ≥90% recipient confirmation within 48h; satisfaction survey returned by ≥50% of cohort.</t>
+          <t>Beneficiary transactions completed in the target window; recipient confirmation and survey targets agreed jointly with partner M&amp;E before pilot start.</t>
         </is>
       </c>
       <c r="E62" s="45" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B63" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Production pilot deployment: dedicated PostgreSQL, monitoring (Sentry + Better Stack), uptime alerting, documented runbook for partner staff.</t>
+          <t>Activity 1 — Production pilot deployment: dedicated PostgreSQL database, production monitoring and uptime alerting, documented runbook for partner staff.</t>
         </is>
       </c>
       <c r="C63" s="46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="D63" s="46" t="inlineStr">
         <is>
-          <t>30-day uptime ≥99%.</t>
+          <t>Operational uptime SLA defined in the partner agreement and met during the pilot window.</t>
         </is>
       </c>
       <c r="E63" s="46" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D64" s="46" t="inlineStr">
         <is>
-          <t>≥25 verified transactions; partner staff operating independently with on-call support.</t>
+          <t>Beneficiaries onboarded successfully; partner staff operating independently with on-call support.</t>
         </is>
       </c>
       <c r="E64" s="46" t="inlineStr">
@@ -2351,22 +2351,22 @@
       </c>
       <c r="C66" s="45" t="inlineStr">
         <is>
-          <t>Shipwreck reports added for the pilot jurisdiction. Hardcoded FX rates replaced with live oracle. Frontend localised to English plus the pilot partner's working language. If the partner's language is Spanish, that counts; otherwise Spanish is not added in this phase.</t>
+          <t>Shipwreck reports added for the pilot jurisdiction. Hardcoded exchange rates replaced with a documented exchange-rate source selected with local advisor input. Frontend localised to English plus the pilot partner's working language. If the partner's language is Spanish, that counts; otherwise Spanish is not added in this phase.</t>
         </is>
       </c>
       <c r="D66" s="45" t="inlineStr">
         <is>
-          <t>i18n strings extracted; 2 languages live (EN + pilot language); native-speaker QA passed; 3 jurisdictions in Shipwreck (US, CO, + pilot); live FX oracle in production.</t>
+          <t>User-facing strings extracted to i18n bundles; pilot language live; native-speaker QA passed; pilot jurisdiction added to Shipwreck templates; documented exchange-rate source in production.</t>
         </is>
       </c>
       <c r="E66" s="45" t="inlineStr">
         <is>
-          <t>i18n bundles, QA reports, per-jurisdiction templates, oracle integration code.</t>
+          <t>i18n bundles, QA reports, per-jurisdiction templates, exchange-rate source integration code and documentation.</t>
         </is>
       </c>
       <c r="F66" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + Carlos Quintero + translation vendor</t>
+          <t>Mateo Daza + Carlos Quintero + translator</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B67" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Extract all user-facing strings using next-intl; engage translation vendor for the pilot-partner language; integrate and QA.</t>
+          <t>Activity 1 — Extract all user-facing strings using a standard i18n library; engage translator for the pilot-partner language; integrate and QA.</t>
         </is>
       </c>
       <c r="C67" s="46" t="inlineStr">
@@ -2410,12 +2410,12 @@
       </c>
       <c r="B68" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Add pilot-jurisdiction Shipwreck template + EU baseline; integrate live FX oracle (Chainlink or CoinGecko API); validate with local advisor.</t>
+          <t>Activity 2 — Add pilot-jurisdiction Shipwreck template + EU baseline; integrate a documented exchange-rate source for Shipwreck reports (selected with local advisor); validate sample PDFs with local advisor.</t>
         </is>
       </c>
       <c r="C68" s="46" t="inlineStr">
         <is>
-          <t>New templates live; live FX in production.</t>
+          <t>New templates live; documented exchange-rate source in production.</t>
         </is>
       </c>
       <c r="D68" s="46" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="E68" s="46" t="inlineStr">
         <is>
-          <t>Code commits, sample PDFs, oracle integration tests.</t>
+          <t>Code commits, sample PDFs, exchange-rate source documentation.</t>
         </is>
       </c>
       <c r="F68" s="46" t="inlineStr">
@@ -2455,12 +2455,12 @@
       </c>
       <c r="C70" s="45" t="inlineStr">
         <is>
-          <t>15 beneficiaries from the pilot cohort + 3-5 partner staff complete structured feedback. Top issues triaged for Q4. All beneficiary research requires ethics/safeguarding clearance and consent/assent instruments approved before data collection begins.</t>
+          <t>a small group of beneficiaries from the pilot cohort + a small group of partner staff complete structured feedback. Top issues triaged for Q4. All beneficiary research requires ethics/safeguarding clearance and consent/assent instruments approved before data collection begins.</t>
         </is>
       </c>
       <c r="D70" s="45" t="inlineStr">
         <is>
-          <t>SUS ≥65; qualitative themes documented; top 5 issues triaged.</t>
+          <t>Usability and acceptance targets agreed with partner M&amp;E before research begins; qualitative themes documented; top 5 issues triaged.</t>
         </is>
       </c>
       <c r="E70" s="45" t="inlineStr">
@@ -2487,12 +2487,12 @@
       </c>
       <c r="C71" s="46" t="inlineStr">
         <is>
-          <t>20 sessions completed.</t>
+          <t>sessions completed (count defined with partner research lead).</t>
         </is>
       </c>
       <c r="D71" s="46" t="inlineStr">
         <is>
-          <t>SUS ≥65; bug list triaged.</t>
+          <t>Acceptance targets met as agreed with partner; bug list triaged.</t>
         </is>
       </c>
       <c r="E71" s="46" t="inlineStr">
@@ -2514,22 +2514,22 @@
       </c>
       <c r="B72" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Targeted first-click tests on Pay and Collect in pilot language.</t>
+          <t>Activity 2 — Targeted usability tests on Pay and Collect flows in the pilot language (unmoderated task completion, captured via standard web-based testing).</t>
         </is>
       </c>
       <c r="C72" s="46" t="inlineStr">
         <is>
-          <t>100+ test responses.</t>
+          <t>Test coverage of Pay and Collect flows as defined with partner UX research.</t>
         </is>
       </c>
       <c r="D72" s="46" t="inlineStr">
         <is>
-          <t>Direct-success rate ≥70%.</t>
+          <t>Targets defined and met as agreed with partner research lead.</t>
         </is>
       </c>
       <c r="E72" s="46" t="inlineStr">
         <is>
-          <t>Maze.co reports.</t>
+          <t>Test reports, anonymised completion logs.</t>
         </is>
       </c>
       <c r="F72" s="46" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="D83" s="47" t="inlineStr">
         <is>
-          <t>Pilot SUS ≥65; native-speaker QA passed.</t>
+          <t>Native-speaker QA passed; usability targets agreed with partner M&amp;E and reported.</t>
         </is>
       </c>
       <c r="E83" s="47" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B85" s="47" t="inlineStr">
         <is>
-          <t>Backend: Pilot environment monitored (≥99% uptime); live FX oracle for Shipwreck; pilot-jurisdiction compliance template added. Note: Q3/Q4 research load (interviews, Maze tests, evaluation, accessibility audit) requires translation vendor, UX research contractor, and partner staff support.</t>
+          <t>Backend: pilot environment monitored with uptime SLA as agreed with partner; documented exchange-rate source integrated for Shipwreck reports; pilot-jurisdiction compliance template added. Note: Q3/Q4 research load (interviews, usability testing, evaluation, accessibility audit) requires partner and advisor support where needed.</t>
         </is>
       </c>
       <c r="C85" s="47" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="D85" s="47" t="inlineStr">
         <is>
-          <t>≥25 verified transactions; advisor sign-offs on compliance templates; uptime ≥99%.</t>
+          <t>Pilot transactions completed as agreed with partner; advisor sign-offs on compliance templates; uptime SLA met.</t>
         </is>
       </c>
       <c r="E85" s="47" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="D88" s="45" t="inlineStr">
         <is>
-          <t>≥75 verified beneficiary transactions; ≥90% recipient confirmation within 48h; SUS ≥70.</t>
+          <t>Expansion cohort transacting successfully; confirmation, satisfaction, and uptime targets agreed jointly with partner M&amp;E before the expansion phase.</t>
         </is>
       </c>
       <c r="E88" s="45" t="inlineStr">
@@ -2935,12 +2935,12 @@
       </c>
       <c r="C90" s="46" t="inlineStr">
         <is>
-          <t>Second cohort transacting with ≤48h confirmation rate ≥90%.</t>
+          <t>Second cohort transacting; targets and reporting cadence defined in the partner agreement.</t>
         </is>
       </c>
       <c r="D90" s="46" t="inlineStr">
         <is>
-          <t>30-day uptime ≥99.5%.</t>
+          <t>Operational uptime SLA met as agreed with partner.</t>
         </is>
       </c>
       <c r="E90" s="46" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="B93" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Engage independent evaluator (e.g., 60 Decibels or local research firm) to assess usability, comprehension, support burden, and partner workflow fit.</t>
+          <t>Activity 1 — Engage independent evaluator (an independent evaluator) to assess usability, comprehension, support burden, and partner workflow fit.</t>
         </is>
       </c>
       <c r="C93" s="46" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D96" s="45" t="inlineStr">
         <is>
-          <t>Docs site live; 2 end-to-end integration tutorials published; ≥1 external developer completes a tutorial.</t>
+          <t>Docs site live; 2 end-to-end integration tutorials published; tutorials available for external developer integration.</t>
         </is>
       </c>
       <c r="E96" s="45" t="inlineStr">
@@ -3178,22 +3178,22 @@
       </c>
       <c r="B100" s="45" t="inlineStr">
         <is>
-          <t>Sustainability roadmap and partner engagement for post-funding viability</t>
+          <t>Sustainability planning and partner engagement for post-funding viability</t>
         </is>
       </c>
       <c r="C100" s="45" t="inlineStr">
         <is>
-          <t>Concrete sustainability plan beyond the funded period: revenue mechanism configured on production; first prospective partners engaged; long-term financial plan delivered.</t>
+          <t>Sustainability planning beyond the funded period: explore partner-supported infrastructure arrangements (waived during pilots), document a long-term plan for continued maintenance, and open conversations with prospective partners. No specific post-funding commitments are made in this proposal.</t>
         </is>
       </c>
       <c r="D100" s="45" t="inlineStr">
         <is>
-          <t>Revenue mechanism configured on production; ≥3 prospective partners in active conversation; sustainability plan delivered.</t>
+          <t>Sustainability plan delivered; prospective partner conversations documented; plan reviewed with Cartagena On Chain and Fabio.</t>
         </is>
       </c>
       <c r="E100" s="45" t="inlineStr">
         <is>
-          <t>Sustainability plan document, prospect-pipeline doc (redacted), on-chain configuration evidence.</t>
+          <t>Sustainability plan document, prospect-pipeline notes (redacted), call notes.</t>
         </is>
       </c>
       <c r="F100" s="45" t="inlineStr">
@@ -3210,22 +3210,22 @@
       </c>
       <c r="B101" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Configure revenue mechanism on production; document operating model.</t>
+          <t>Activity 1 — Document sustainability approach and partner support model; share with Cartagena On Chain leadership for review.</t>
         </is>
       </c>
       <c r="C101" s="46" t="inlineStr">
         <is>
-          <t>Revenue mechanism live.</t>
+          <t>Sustainability plan documented and reviewed.</t>
         </is>
       </c>
       <c r="D101" s="46" t="inlineStr">
         <is>
-          <t>Production configuration verified on-chain.</t>
+          <t>Plan signed off by Cartagena On Chain.</t>
         </is>
       </c>
       <c r="E101" s="46" t="inlineStr">
         <is>
-          <t>Configuration evidence, tx hashes.</t>
+          <t>Sustainability plan document.</t>
         </is>
       </c>
       <c r="F101" s="46" t="inlineStr">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="B102" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Open conversations with 3-5 organisations (NGOs, foundations, donor platforms) about paid ASP-attestation tiers; document interest and objections.</t>
+          <t>Activity 2 — Open conversations with a small number of organisations   about ongoing collaboration; document interest and feedback.</t>
         </is>
       </c>
       <c r="C102" s="46" t="inlineStr">
         <is>
-          <t>3-5 conversations completed.</t>
+          <t>Conversations documented with feedback.</t>
         </is>
       </c>
       <c r="D102" s="46" t="inlineStr">
@@ -3287,22 +3287,22 @@
       </c>
       <c r="C104" s="45" t="inlineStr">
         <is>
-          <t>Closing round of validation across personas + accessibility conformance pass. Research sessions, Maze testing, and accessibility audit require vendor and partner support; this dependency is built into the Q4 timeline and staffing plan.</t>
+          <t>Closing round of validation across personas plus accessibility conformance pass. Research sessions and accessibility audit require vendor and partner support; this dependency is acknowledged in the partner agreement.</t>
         </is>
       </c>
       <c r="D104" s="45" t="inlineStr">
         <is>
-          <t>SUS ≥75 across personas; WCAG 2.1 AA conformance on the key user flows.</t>
+          <t>Validation targets agreed with partner research lead; WCAG 2.1 AA conformance on the key user flows (Setup, Pay, Collect, Reports).</t>
         </is>
       </c>
       <c r="E104" s="45" t="inlineStr">
         <is>
-          <t>Recordings, SUS scores, accessibility audit report.</t>
+          <t>Recordings, usability score, accessibility audit report.</t>
         </is>
       </c>
       <c r="F104" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + external accessibility auditor</t>
+          <t>Mateo Daza + accessibility specialist</t>
         </is>
       </c>
     </row>
@@ -3319,12 +3319,12 @@
       </c>
       <c r="C105" s="46" t="inlineStr">
         <is>
-          <t>30 sessions.</t>
+          <t>Number of sessions defined with partner UX research; synthesis report delivered.</t>
         </is>
       </c>
       <c r="D105" s="46" t="inlineStr">
         <is>
-          <t>SUS ≥75.</t>
+          <t>Targets agreed in advance with partner; bug list triaged.</t>
         </is>
       </c>
       <c r="E105" s="46" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B106" s="46" t="inlineStr">
         <is>
-          <t>Accessibility audit. Third-party WCAG 2.1 AA audit on Setup, Pay, Collect, Reports.</t>
+          <t>Accessibility audit. WCAG 2.1 AA audit on Setup, Pay, Collect, Reports.</t>
         </is>
       </c>
       <c r="C106" s="46" t="inlineStr">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="E106" s="46" t="inlineStr">
         <is>
-          <t>Audit report, axe-core CI results.</t>
+          <t>Audit report.</t>
         </is>
       </c>
       <c r="F106" s="46" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="D109" s="47" t="inlineStr">
         <is>
-          <t>SUS ≥70; accessibility audit passed.</t>
+          <t>Validation targets agreed with partner and met; accessibility audit passed.</t>
         </is>
       </c>
       <c r="E109" s="47" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B111" s="47" t="inlineStr">
         <is>
-          <t>Backend: Implementation and usability evaluation published with partner; sustainability roadmap with revenue mechanism live and first prospects engaged; dev docs at docs.galeon.finance.</t>
+          <t>Backend: Implementation and usability evaluation published with partner; sustainability plan delivered; developer documentation at docs.galeon.finance.</t>
         </is>
       </c>
       <c r="C111" s="47" t="inlineStr">
@@ -3448,12 +3448,12 @@
       </c>
       <c r="D111" s="47" t="inlineStr">
         <is>
-          <t>Evaluation report published; revenue mechanism live; docs site live.</t>
+          <t>Evaluation report published; sustainability plan delivered; docs site live.</t>
         </is>
       </c>
       <c r="E111" s="47" t="inlineStr">
         <is>
-          <t>Sustainability plan, prospect pipeline, implementation-evaluation.pdf.</t>
+          <t>Sustainability plan, prospect notes, implementation-evaluation.pdf.</t>
         </is>
       </c>
       <c r="F111" s="48" t="inlineStr">
@@ -3554,7 +3554,7 @@
       <c r="A121" s="13" t="n"/>
       <c r="B121" s="50" t="inlineStr">
         <is>
-          <t>4. Embedded email-based wallet (Privy) + account abstraction + mobile-first UX for non-crypto-literate beneficiaries (no seed phrases, no gas, mobile-optimised).</t>
+          <t>4. Embedded email-based wallet onboarding (Privy or equivalent) with mobile-first UX for non-crypto-literate beneficiaries; gas-simplification options evaluated and implemented where supported by the provider.</t>
         </is>
       </c>
       <c r="C121" s="17" t="n"/>
@@ -3602,7 +3602,7 @@
       <c r="A125" s="13" t="n"/>
       <c r="B125" s="50" t="inlineStr">
         <is>
-          <t>(iii) Embedded-wallet + account-abstraction onboarding integration and mobile-first low-literacy UI components — MIT.</t>
+          <t>(iii) Embedded-wallet onboarding integration and mobile-first low-literacy UI components — MIT.</t>
         </is>
       </c>
       <c r="C125" s="17" t="n"/>
@@ -3638,7 +3638,7 @@
       <c r="A128" s="13" t="n"/>
       <c r="B128" s="52" t="inlineStr">
         <is>
-          <t>None. Every new component developed during the UNICEF-funded period will be released under an OSI-approved permissive licence. Licensing follows the existing repo convention: MIT for applications and libraries (apps/web, apps/api, apps/indexer, packages/stealth, packages/config, packages/types, packages/eslint-config); Apache-2.0 for smart contracts and pool SDK (packages/contracts, packages/pool — inherited from 0xbow upstream). The repository is already public. The only non-public elements are: (a) operational pilot configuration data (kept private for beneficiary safety, not as IP); (b) commercial agreements with paying ASP-attestation customers (contracts, not code).</t>
+          <t>None. Every new component developed during the UNICEF-funded period will be released under an OSI-approved permissive licence. Licensing follows the existing repo convention: MIT for applications and libraries (apps/web, apps/api, apps/indexer, packages/stealth, packages/config, packages/types, packages/eslint-config); Apache-2.0 for smart contracts and pool SDK (packages/contracts, packages/pool — inherited from 0xbow upstream). The repository is already public. The only non-public elements are operational pilot configuration data and partner-specific legal/operational agreements, kept private for beneficiary safety and compliance — not as proprietary software or Project IP.</t>
         </is>
       </c>
       <c r="C128" s="17" t="n"/>

</xml_diff>

<commit_message>
docs: finalize UNICEF submission package
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_DataPlan.xlsx
+++ b/Galeon_UNICEF_DataPlan.xlsx
@@ -2366,7 +2366,7 @@
       </c>
       <c r="F66" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + Carlos Quintero + translator</t>
+          <t>Mateo Daza + Carlos Quintero + partner or in-house translation support</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B67" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Extract all user-facing strings using a standard i18n library; engage translator for the pilot-partner language; integrate and QA.</t>
+          <t>Activity 1 — Extract all user-facing strings using a standard i18n library; translation handled by partner or in-house; specific pilot-language needs and any additional translation support are confirmed jointly with partner before localisation.</t>
         </is>
       </c>
       <c r="C67" s="46" t="inlineStr">
@@ -2975,12 +2975,12 @@
       </c>
       <c r="C92" s="45" t="inlineStr">
         <is>
-          <t>External evaluator assesses: usability (task completion, comprehension), support burden (incidents per beneficiary, escalation rate), partner workflow fit (staff time per cohort, runbook adherence), and incident rate. Ethics/safeguarding clearance renewed for expanded cohort. Joint evaluation report with partner.</t>
+          <t>Implementation and usability evaluation co-conducted with the partner M&amp;E lead: usability (task completion, comprehension), support burden (incidents per beneficiary, escalation rate), partner workflow fit (staff time per cohort, runbook adherence), and incident rate. Ethics/safeguarding clearance renewed for expanded cohort. Joint evaluation report with partner.</t>
         </is>
       </c>
       <c r="D92" s="45" t="inlineStr">
         <is>
-          <t>External evaluator report delivered; measures usability, comprehension, support burden, incident rate, and partner workflow fit.</t>
+          <t>Evaluation report delivered jointly with partner M&amp;E lead; covers usability, comprehension, support burden, incident rate, and partner workflow fit.</t>
         </is>
       </c>
       <c r="E92" s="45" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="F92" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + Fabio Anaya + external evaluator + partner M&amp;E lead</t>
+          <t>Mateo Daza + Fabio Anaya + Juan David Correa + partner M&amp;E lead</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="B93" s="46" t="inlineStr">
         <is>
-          <t>Activity 1 — Engage independent evaluator (an independent evaluator) to assess usability, comprehension, support burden, and partner workflow fit.</t>
+          <t>Activity 1 — Co-conduct evaluation with the partner M&amp;E lead following the partner's monitoring methodology; produce shared assessment instruments and data-collection plan.</t>
         </is>
       </c>
       <c r="C93" s="46" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="F93" s="46" t="inlineStr">
         <is>
-          <t>Mateo Daza + evaluator</t>
+          <t>Mateo Daza + partner M&amp;E lead</t>
         </is>
       </c>
     </row>
@@ -3287,12 +3287,12 @@
       </c>
       <c r="C104" s="45" t="inlineStr">
         <is>
-          <t>Closing round of validation across personas plus accessibility conformance pass. Research sessions and accessibility audit require vendor and partner support; this dependency is acknowledged in the partner agreement.</t>
+          <t>Closing round of validation across personas plus accessibility conformance review. Research sessions co-conducted with partner; accessibility conformance reviewed in-house using standard tooling.</t>
         </is>
       </c>
       <c r="D104" s="45" t="inlineStr">
         <is>
-          <t>Validation targets agreed with partner research lead; WCAG 2.1 AA conformance on the key user flows (Setup, Pay, Collect, Reports).</t>
+          <t>Validation completed jointly with partner research lead; WCAG 2.1 AA conformance on the key user flows (Setup, Pay, Collect, Reports), documented in-house.</t>
         </is>
       </c>
       <c r="E104" s="45" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="F104" s="45" t="inlineStr">
         <is>
-          <t>Mateo Daza + accessibility specialist</t>
+          <t>Mateo Daza</t>
         </is>
       </c>
     </row>
@@ -3346,22 +3346,22 @@
       </c>
       <c r="B106" s="46" t="inlineStr">
         <is>
-          <t>Accessibility audit. WCAG 2.1 AA audit on Setup, Pay, Collect, Reports.</t>
+          <t>Activity 2 — Accessibility conformance review on Setup, Pay, Collect, Reports. Conducted in-house using standard accessibility tooling and the WCAG 2.1 AA checklist; methodology and findings documented and published with the implementation evaluation.</t>
         </is>
       </c>
       <c r="C106" s="46" t="inlineStr">
         <is>
-          <t>Conformance achieved on key flows.</t>
+          <t>Conformance review completed on key user flows.</t>
         </is>
       </c>
       <c r="D106" s="46" t="inlineStr">
         <is>
-          <t>Conformance report passed.</t>
+          <t>WCAG 2.1 AA self-conformance documented; remediations applied.</t>
         </is>
       </c>
       <c r="E106" s="46" t="inlineStr">
         <is>
-          <t>Audit report.</t>
+          <t>Conformance review document, remediation diff.</t>
         </is>
       </c>
       <c r="F106" s="46" t="inlineStr">

</xml_diff>

<commit_message>
fix: removing format mentions
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_DataPlan.xlsx
+++ b/Galeon_UNICEF_DataPlan.xlsx
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E13" s="46" t="inlineStr">
         <is>
-          <t>Git tag, threat-model.md, modifications-diff.md.</t>
+          <t>Git tag, threat model document, custom-modifications diff.</t>
         </is>
       </c>
       <c r="F13" s="46" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="E15" s="45" t="inlineStr">
         <is>
-          <t>Discovery notes (with consent), partner-fit matrix, LOI document, operational-dependency-model.md.</t>
+          <t>Discovery notes (with consent), partner-fit matrix, LOI document, operational dependency model document.</t>
         </is>
       </c>
       <c r="F15" s="45" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="E17" s="46" t="inlineStr">
         <is>
-          <t>LOI PDF, operational-dependency-model.md.</t>
+          <t>LOI PDF, operational dependency model document.</t>
         </is>
       </c>
       <c r="F17" s="46" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="E37" s="46" t="inlineStr">
         <is>
-          <t>ASP-policy.md, IPFS CIDs, on-chain tx hashes.</t>
+          <t>ASP policy document, IPFS CIDs, on-chain tx hashes.</t>
         </is>
       </c>
       <c r="F37" s="46" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="E47" s="45" t="inlineStr">
         <is>
-          <t>CONTRIBUTING.md, CODE_OF_CONDUCT.md, secrets-scan report, UNICEF attribution diff, repository activity log.</t>
+          <t>Public-repo URL, contributing guide, code of conduct, secrets-scan report, UNICEF attribution diff, repository activity log.</t>
         </is>
       </c>
       <c r="F47" s="45" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B49" s="46" t="inlineStr">
         <is>
-          <t>Activity 2 — Publish CONTRIBUTING.md, CODE_OF_CONDUCT.md, and governance notes; apply UNICEF Innovation Fund attribution to the repository per contractual terms; publish an open-source community announcement.</t>
+          <t>Activity 2 — Apply UNICEF Innovation Fund attribution to the repository per contract terms; publish a basic contributing guide and code of conduct for external contributors.</t>
         </is>
       </c>
       <c r="C49" s="46" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="E49" s="46" t="inlineStr">
         <is>
-          <t>CONTRIBUTING.md, CODE_OF_CONDUCT.md, attribution commit, announcement post.</t>
+          <t>Contributing guide, code of conduct, attribution commit, announcement post.</t>
         </is>
       </c>
       <c r="F49" s="46" t="inlineStr">

</xml_diff>

<commit_message>
fix: unicef docs final polish
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_DataPlan.xlsx
+++ b/Galeon_UNICEF_DataPlan.xlsx
@@ -2398,7 +2398,7 @@
       </c>
       <c r="F67" s="46" t="inlineStr">
         <is>
-          <t>Mateo Daza + vendor</t>
+          <t>Mateo Daza + partner or in-house translation support</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B85" s="47" t="inlineStr">
         <is>
-          <t>Backend: pilot environment monitored with uptime SLA as agreed with partner; documented exchange-rate source integrated for Shipwreck reports; pilot-jurisdiction compliance template added. Note: Q3/Q4 research load (interviews, usability testing, evaluation, accessibility audit) requires partner and advisor support where needed.</t>
+          <t>Backend: pilot environment monitored with uptime SLA as agreed with partner; documented exchange-rate source integrated for Shipwreck reports; pilot-jurisdiction compliance template added. Note: Q3/Q4 research load (interviews, usability testing, evaluation, accessibility conformance review) requires partner and advisor support where needed.</t>
         </is>
       </c>
       <c r="C85" s="47" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B92" s="45" t="inlineStr">
         <is>
-          <t>Independent implementation and usability evaluation</t>
+          <t>Implementation and usability evaluation co-conducted with partner M&amp;E lead</t>
         </is>
       </c>
       <c r="C92" s="45" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="E104" s="45" t="inlineStr">
         <is>
-          <t>Recordings, usability score, accessibility audit report.</t>
+          <t>Recordings, usability score, accessibility conformance review report.</t>
         </is>
       </c>
       <c r="F104" s="45" t="inlineStr">
@@ -3408,12 +3408,12 @@
       </c>
       <c r="D109" s="47" t="inlineStr">
         <is>
-          <t>Validation targets agreed with partner and met; accessibility audit passed.</t>
+          <t>Validation targets agreed with partner and met; accessibility conformance review completed.</t>
         </is>
       </c>
       <c r="E109" s="47" t="inlineStr">
         <is>
-          <t>Public repo, docs site, accessibility-report.pdf.</t>
+          <t>Public repo, docs site, accessibility-conformance-review.pdf.</t>
         </is>
       </c>
       <c r="F109" s="48" t="inlineStr">

</xml_diff>